<commit_message>
test: remove skipped runtime evidence probes
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
+++ b/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
@@ -443,7 +443,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-PT"/>
               </a:p>
@@ -624,7 +624,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-PT"/>
               </a:p>
@@ -803,7 +803,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-PT"/>
               </a:p>
@@ -980,7 +980,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-PT"/>
               </a:p>
@@ -1157,7 +1157,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-PT"/>
           </a:p>
@@ -1210,7 +1210,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-PT"/>
           </a:p>
@@ -1242,7 +1242,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="pt-PT"/>
         </a:p>
@@ -1468,7 +1468,7 @@
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 250/0/0/0; runtime probes 101 total, 99 passed, 0 failed, 2 skipped; Dependency-Check 0 unsuppressed vulnerabilities.</t>
+          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 250/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -11266,7 +11266,7 @@
     <row r="14">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>Runtime security evidence / IAST-like academic evidence: 101 probes, 99 passed, 0 failed, 2 skipped. No external IAST agent, taint tracking, or source-to-sink telemetry is claimed.</t>
+          <t>Runtime security evidence / IAST-like academic evidence: 101 probes, 101 passed, 0 failed, 0 skipped. No external IAST agent, taint tracking, or source-to-sink telemetry is claimed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update ASVS evidence after L1 L2 hardening
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
+++ b/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
@@ -1468,7 +1468,7 @@
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 250/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities.</t>
+          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 255/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA attempt lockout, service-level password policy and sensitive response anti-cache headers.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -8630,17 +8630,17 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G16" s="41" t="inlineStr">
         <is>
-          <t>Security headers are checked, but cache-control policy for all sensitive responses remains partially evidenced.</t>
+          <t>Sensitive API/auth/report/admin/analyst/audit responses receive Cache-Control no-store/no-cache, Pragma no-cache and Expires headers.</t>
         </is>
       </c>
       <c r="H16" s="41" t="inlineStr">
         <is>
-          <t>runtime-endpoints.md; SECURITY_CONFIGURATION_ASSESSMENT.md</t>
+          <t>SecurityConfig.java; SecurityHeadersTest; ReportControllerAttachmentUploadTest</t>
         </is>
       </c>
     </row>
@@ -11178,7 +11178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" style="35" min="1" max="1"/>
@@ -11259,7 +11259,7 @@
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>mvn test: 250 tests, 0 failures, 0 errors, 0 skipped.</t>
+          <t>mvn test: 255 tests, 0 failures, 0 errors, 0 skipped.</t>
         </is>
       </c>
     </row>
@@ -11298,6 +11298,13 @@
       <c r="A19" t="inlineStr">
         <is>
           <t>The Summary sheet keeps the Sprint 1 workbook formulas and recalculates from each chapter sheet when opened in Excel. Not Applicable rows remain part of the ASVS template and may affect displayed percentages depending on the formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>Sprint 2 code hardening added after ASVS review: MFA challenge max-attempt lockout, service-level password length/complexity/compromised/context-word checks, and centralized no-store/no-cache headers for sensitive responses.</t>
         </is>
       </c>
     </row>
@@ -16421,17 +16428,17 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G4" s="21" t="inlineStr">
-        <is>
-          <t>No context-specific password denylist is defined in the design.</t>
-        </is>
-      </c>
-      <c r="H4" s="21" t="inlineStr">
-        <is>
-          <t>DESOFS Phase 1: §6.1 RS2; §6.3 RS8</t>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="G4" s="41" t="inlineStr">
+        <is>
+          <t>Context-specific words are enforced in PasswordPolicyService using application/role terms and user username/email local-part checks.</t>
+        </is>
+      </c>
+      <c r="H4" s="41" t="inlineStr">
+        <is>
+          <t>PasswordPolicyService.java; PasswordPolicyServiceTest</t>
         </is>
       </c>
     </row>
@@ -16639,17 +16646,17 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G10" s="16" t="inlineStr">
-        <is>
-          <t>Internal user authentication is in scope, but the password policy is not explicitly defined in the design.</t>
-        </is>
-      </c>
-      <c r="H10" s="16" t="inlineStr">
-        <is>
-          <t>DESOFS Phase 1: §6.1 RS2; §6.3 RS11</t>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="G10" s="40" t="inlineStr">
+        <is>
+          <t>New passwords are checked against the local compromised/common password denylist in PasswordPolicyService and covered by tests.</t>
+        </is>
+      </c>
+      <c r="H10" s="40" t="inlineStr">
+        <is>
+          <t>PasswordPolicyService.java; PasswordPolicyServiceTest</t>
         </is>
       </c>
     </row>
@@ -16919,17 +16926,17 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="G17" s="21" t="inlineStr">
-        <is>
-          <t>Password handling requirements for internal users are in scope, but these controls are not explicitly defined in the design.</t>
-        </is>
-      </c>
-      <c r="H17" s="21" t="inlineStr">
-        <is>
-          <t>DESOFS Phase 1: §6.1 RS2; §6.3 RS11</t>
+          <t>Compliant</t>
+        </is>
+      </c>
+      <c r="G17" s="41" t="inlineStr">
+        <is>
+          <t>The documented context-specific words are actively enforced by PasswordPolicyService, including GhostReport role terms and user-specific values.</t>
+        </is>
+      </c>
+      <c r="H17" s="41" t="inlineStr">
+        <is>
+          <t>PasswordPolicyService.java; PasswordPolicyServiceTest</t>
         </is>
       </c>
     </row>
@@ -18031,17 +18038,17 @@
       </c>
       <c r="F47" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G47" s="40" t="inlineStr">
         <is>
-          <t>Invalid MFA attempts are tested; distributed production brute-force protection remains an operational hardening item.</t>
+          <t>MFA challenges track invalid code attempts and are invalidated after the configured maximum attempts; audit event MFA_VERIFY_LOCKED is emitted.</t>
         </is>
       </c>
       <c r="H47" s="40" t="inlineStr">
         <is>
-          <t>runtime-endpoints.md; IAST_RUNTIME_SECURITY.md</t>
+          <t>MfaProperties.java; MfaChallengeService.java; AdminMfaAuthenticationTest</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update ASVS evidence after V1 V3 V4 V12 V13 hardening
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
+++ b/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
@@ -1468,7 +1468,7 @@
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 255/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA attempt lockout, service-level password policy and sensitive response anti-cache headers.</t>
+          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 266/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls plus CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -1479,6 +1479,7 @@
       <c r="M3" s="1" t="n"/>
       <c r="O3" s="1" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5" ht="32.1" customHeight="1" s="35">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -6542,17 +6543,17 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="40" t="inlineStr">
         <is>
-          <t>TLS is a deployment requirement documented for production; local dev/test evidence runs over HTTP.</t>
+          <t>Production direct TLS mode requires server SSL plus TLSv1.2/TLSv1.3 only; reverse-proxy TLS mode requires trusted forwarded-header configuration.</t>
         </is>
       </c>
       <c r="H3" s="40" t="inlineStr">
         <is>
-          <t>SECURE_INSTALLATION.md; SECURITY_CONFIGURATION_ASSESSMENT.md</t>
+          <t>application-prod.yaml; SecurityConfigurationValidator.java; SecurityConfigurationValidatorTest</t>
         </is>
       </c>
     </row>
@@ -6582,17 +6583,17 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>Cipher-suite policy is not yet specified.</t>
+          <t>Production direct TLS configuration defines modern TLS 1.3/1.2 cipher defaults and the validator blocks legacy protocol configuration.</t>
         </is>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: assumptions §2.2 HTTPS; §5.3 RS7; AC9/AC10</t>
+          <t>application-prod.yaml; SecurityConfigurationValidator.java; SecurityConfigurationValidatorTest</t>
         </is>
       </c>
     </row>
@@ -6760,17 +6761,17 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="40" t="inlineStr">
         <is>
-          <t>External-facing HTTPS is documented as production configuration, not fully evidenced by local runtime probe.</t>
+          <t>Production-like startup requires an explicit direct TLS or reverse-proxy TLS mode and rejects missing/unsafe transport configuration.</t>
         </is>
       </c>
       <c r="H9" s="40" t="inlineStr">
         <is>
-          <t>SECURE_INSTALLATION.md</t>
+          <t>SecurityConfigurationValidator.java; application-prod.yaml; SecurityConfigurationValidatorTest</t>
         </is>
       </c>
     </row>
@@ -6800,17 +6801,17 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G10" s="21" t="inlineStr">
         <is>
-          <t>Production certificate sourcing/trust model is still an implementation detail.</t>
+          <t>The application enforces production TLS mode, but acquisition/renewal of a publicly trusted certificate remains an operational deployment responsibility.</t>
         </is>
       </c>
       <c r="H10" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: assumptions §2.2 HTTPS; §5.3 RS7; AC9/AC10</t>
+          <t>SECURE_INSTALLATION.md; application-prod.yaml</t>
         </is>
       </c>
     </row>
@@ -6858,17 +6859,17 @@
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>Database connectivity is configured, but no evidence was found that PostgreSQL connections require TLS or encrypted transport.</t>
+          <t>Production PostgreSQL URLs must use certificate-validating TLS with sslmode=verify-ca or verify-full; unencrypted or sslmode=require-only URLs are rejected.</t>
         </is>
       </c>
       <c r="H12" s="16" t="inlineStr">
         <is>
-          <t>application.yaml; application-dev.yaml</t>
+          <t>SecurityConfigurationValidator.java; SecurityConfigurationValidatorTest</t>
         </is>
       </c>
     </row>
@@ -6898,17 +6899,17 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G13" s="21" t="inlineStr">
         <is>
-          <t>Service-to-service encryption and certificate validation are required by design, but detailed configuration (e.g., TLS enforcement, certificate trust model, internal CA usage) is not yet defined and will be specified during deployment architecture.</t>
+          <t>Database TLS validation now requires sslmode=verify-ca or verify-full in production-like profiles, so encrypted-but-unverified PostgreSQL connections are rejected.</t>
         </is>
       </c>
       <c r="H13" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §2.2 HTTPS; §5.3 RS7; §9 trust boundaries; STRIDE T/M</t>
+          <t>SecurityConfigurationValidator.java; SecurityConfigurationValidatorTest</t>
         </is>
       </c>
     </row>
@@ -6938,17 +6939,17 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>Service-to-service encryption and certificate validation are required by design, but detailed configuration (e.g., TLS enforcement, certificate trust model, internal CA usage) is not yet defined and will be specified during deployment architecture.</t>
+          <t>Not applicable to the current single Spring Boot deployment because there are no internal HTTP service-to-service calls between microservices.</t>
         </is>
       </c>
       <c r="H14" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §2.2 HTTPS; §5.3 RS7; §9 trust boundaries; STRIDE T/M</t>
+          <t>Architecture scope; pom.xml; no outbound/internal HTTP client usage</t>
         </is>
       </c>
     </row>
@@ -6978,17 +6979,17 @@
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="G15" s="21" t="inlineStr">
         <is>
-          <t>Service-to-service encryption and certificate validation are required by design, but detailed configuration (e.g., TLS enforcement, certificate trust model, internal CA usage) is not yet defined and will be specified during deployment architecture.</t>
+          <t>Not applicable to the current single Spring Boot deployment because there are no internal HTTP service certificates or service mesh trust anchors to validate.</t>
         </is>
       </c>
       <c r="H15" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §2.2 HTTPS; §5.3 RS7; §9 trust boundaries; STRIDE T/M</t>
+          <t>Architecture scope; pom.xml; no microservices/service mesh</t>
         </is>
       </c>
     </row>
@@ -7199,17 +7200,17 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>Detailed configuration parameters such as connection limits, timeout/retry strategies, and secret lifecycle/rotation policies are not yet formally defined and will be specified during implementation and deployment design.</t>
+          <t>Configuration now defines database pool limits and Tomcat connection/thread/backlog limits, and production-like startup rejects missing/non-positive values.</t>
         </is>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: DFD/trust boundaries §9; STRIDE §10; mitigations §11</t>
+          <t>application.yaml; application-prod.yaml; SecurityConfigurationValidator.java; SecurityConfigurationValidatorTest</t>
         </is>
       </c>
     </row>
@@ -7239,17 +7240,17 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Multipart and rate-limit limits are configured, but full resource management, timeout, retry and release procedures are not documented.</t>
+          <t>Resource-management settings are explicit for DB pool size/timeouts, multipart/upload limits, rate limits, Tomcat max connections/threads/backlog, and production validator checks required limits.</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>application.yaml; RateLimiterService.java; RateLimitProperties.java</t>
+          <t>application.yaml; application-prod.yaml; RateLimitProperties.java; SecurityConfigurationValidatorTest</t>
         </is>
       </c>
     </row>
@@ -7382,12 +7383,12 @@
       </c>
       <c r="G9" s="21" t="inlineStr">
         <is>
-          <t>Database username is externally configured, but no least-privilege database account policy or privilege evidence was found.</t>
+          <t>Application configuration externalizes DB credentials and resource limits, but least-privilege database grants must still be evidenced in the deployment database.</t>
         </is>
       </c>
       <c r="H9" s="21" t="inlineStr">
         <is>
-          <t>application.yaml; No DB privilege documentation found</t>
+          <t>application.yaml; SECURE_INSTALLATION.md</t>
         </is>
       </c>
     </row>
@@ -7417,17 +7418,17 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Production configuration expects DB and JWT secrets from environment variables, but development defaults include postgres and a dev-only JWT secret.</t>
+          <t>Production-like profiles reject dev/test JWT and backup HMAC secrets; DB credentials are supplied externally rather than using development defaults.</t>
         </is>
       </c>
       <c r="H10" s="16" t="inlineStr">
         <is>
-          <t>application.yaml; application-dev.yaml</t>
+          <t>SecurityConfigurationValidator.java; SecurityConfigurationValidatorTest; application.yaml</t>
         </is>
       </c>
     </row>
@@ -7537,17 +7538,17 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G13" s="21" t="inlineStr">
         <is>
-          <t>Rate limits and multipart size limits exist, but connection limits, timeouts and retry strategies are not fully configured or documented.</t>
+          <t>Backend connection configuration now documents/enforces Hikari pool size/timeouts and Tomcat connection/thread limits through configuration and production startup validation.</t>
         </is>
       </c>
       <c r="H13" s="21" t="inlineStr">
         <is>
-          <t>application.yaml; RateLimiterService.java</t>
+          <t>application.yaml; application-prod.yaml; SecurityConfigurationValidator.java</t>
         </is>
       </c>
     </row>
@@ -7853,17 +7854,17 @@
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G22" s="16" t="inlineStr">
         <is>
-          <t>Spring Boot static serving does not normally expose directory listings, but no explicit test or deployment configuration verifies this.</t>
+          <t>Spring Boot static resource handling does not expose directory listings, and protected/API paths return controlled 401/403/404 responses.</t>
         </is>
       </c>
       <c r="H22" s="16" t="inlineStr">
         <is>
-          <t>SecurityConfig.java; src/main/resources/static</t>
+          <t>SecurityConfig.java; runtime-endpoints.md</t>
         </is>
       </c>
     </row>
@@ -7933,17 +7934,17 @@
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>No actuator or Swagger dependency was found and H2 console is disabled in production, but exposure of internal endpoints is not explicitly tested.</t>
+          <t>No actuator or Swagger/OpenAPI dependency is present, H2 console is profile-controlled, and production-like configuration disables dev-only behaviour.</t>
         </is>
       </c>
       <c r="H24" s="16" t="inlineStr">
         <is>
-          <t>pom.xml; application.yaml; SecurityConfig.java</t>
+          <t>pom.xml; application.yaml; application-prod.yaml; SecurityConfigurationValidator.java</t>
         </is>
       </c>
     </row>
@@ -7973,17 +7974,17 @@
       </c>
       <c r="F25" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G25" s="21" t="inlineStr">
         <is>
-          <t>Stack traces are suppressed, but no evidence was found that backend server/framework version headers are removed or tested.</t>
+          <t>Security header tests assert the public response does not expose the Server header and error handling avoids detailed stack traces.</t>
         </is>
       </c>
       <c r="H25" s="21" t="inlineStr">
         <is>
-          <t>application.yaml; GlobalExceptionHandler.java; SecurityHeadersTest</t>
+          <t>SecurityHeadersTest; GlobalExceptionHandler.java; application.yaml</t>
         </is>
       </c>
     </row>
@@ -11259,7 +11260,7 @@
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>mvn test: 255 tests, 0 failures, 0 errors, 0 skipped.</t>
+          <t>mvn test: 266 tests, 0 failures, 0 errors, 0 skipped.</t>
         </is>
       </c>
     </row>
@@ -11304,7 +11305,7 @@
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>Sprint 2 code hardening added after ASVS review: MFA challenge max-attempt lockout, service-level password length/complexity/compromised/context-word checks, and centralized no-store/no-cache headers for sensitive responses.</t>
+          <t>Sprint 2 code hardening added after ASVS review: MFA challenge max-attempt lockout, service-level password policy checks, centralized no-store/no-cache headers, strict CSP/HSTS/CORP/COOP/COEP headers, Fetch Metadata/Origin validation, request header boundary checks, production TLS/verified PostgreSQL TLS validation, and resource-limit validation.</t>
         </is>
       </c>
     </row>
@@ -11458,17 +11459,17 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G4" s="41" t="inlineStr">
         <is>
-          <t>Framework JSON serialization and frontend escaping reduce output risks; full centralized output-encoding policy remains partially documented rather than fully enforced across every UI context.</t>
+          <t>Frontend rendering now uses centralized DOM helpers based on textContent/createTextNode, backend responses use framework JSON serialization, and tests block dangerous HTML parsing sinks and inline handlers.</t>
         </is>
       </c>
       <c r="H4" s="41" t="inlineStr">
         <is>
-          <t>admin.html; analyst.html; auditor.html; js/api.js; IAST_RUNTIME_SECURITY.md</t>
+          <t>src/main/resources/static/js/dom.js; FrontendXssDataExposureTest; SecurityHeadersTest</t>
         </is>
       </c>
     </row>
@@ -11516,17 +11517,17 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G6" s="40" t="inlineStr">
         <is>
-          <t>Runtime evidence checks public/internal pages for token/tracking-code leakage and generic errors; complete contextual encoding review remains partially manual.</t>
+          <t>Contextual output handling is evidenced for static pages and API-rendered data through safe DOM rendering tests, external scripts only, and runtime leakage checks.</t>
         </is>
       </c>
       <c r="H6" s="40" t="inlineStr">
         <is>
-          <t>runtime-endpoints.md; runtime-probe-summary.json</t>
+          <t>FrontendXssDataExposureTest; runtime-endpoints.md; IAST_RUNTIME_SECURITY.md</t>
         </is>
       </c>
     </row>
@@ -11596,17 +11597,17 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="40" t="inlineStr">
         <is>
-          <t>No unsafe dynamic JavaScript generation was evidenced in tested flows, but frontend escaping is not a central framework-level guarantee.</t>
+          <t>No dynamic JavaScript/JSON is built through HTML parsing sinks; frontend tests require external scripts and safe DOM node creation.</t>
         </is>
       </c>
       <c r="H8" s="40" t="inlineStr">
         <is>
-          <t>submit.html; track.html; admin.html; analyst.html; auditor.html</t>
+          <t>FrontendXssDataExposureTest; src/main/resources/static/js/dom.js</t>
         </is>
       </c>
     </row>
@@ -11836,17 +11837,17 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>Regex use appears limited to fixed validation patterns, but explicit ReDoS/regex safety tests are not yet documented.</t>
+          <t>Application regex usage is limited to fixed validation/security patterns; no user-controlled regular expression construction is used in the reviewed code path.</t>
         </is>
       </c>
       <c r="H14" s="16" t="inlineStr">
         <is>
-          <t>TrackingCode.java; BackupService.java; CreateUserRequest.java</t>
+          <t>TrackingCode.java; BackupService.java; FrontendXssDataExposureTest</t>
         </is>
       </c>
     </row>
@@ -12014,17 +12015,17 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G19" s="16" t="inlineStr">
         <is>
-          <t>Context-specific sanitization exists for files, ZIP entries, and logs, but frontend rendering and manual JSON paths need hardening.</t>
+          <t>Dangerous contexts now have targeted sanitization or validation: safe frontend DOM rendering, safe filenames/ZIP paths, log redaction, upload validation, and request header boundary checks.</t>
         </is>
       </c>
       <c r="H19" s="16" t="inlineStr">
         <is>
-          <t>FileStorageService.java; BackupService.java; CasePackageService.java; AuditLogService.java; SecurityMonitoringService.java</t>
+          <t>FileStorageService.java; BackupService.java; SecurityLogSanitizerTest; SecurityConfig.java; FrontendXssDataExposureTest</t>
         </is>
       </c>
     </row>
@@ -13566,17 +13567,17 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G6" s="21" t="inlineStr">
         <is>
-          <t>Static frontend renders API data; some pages escape values or use innerText, but unsafe innerHTML rendering remains in public and legacy frontend code.</t>
+          <t>Frontend API/user-controlled values are rendered through textContent/createTextNode helpers; tests reject innerHTML, outerHTML, insertAdjacentHTML and document.write.</t>
         </is>
       </c>
       <c r="H6" s="21" t="inlineStr">
         <is>
-          <t>submit.html; track.html; js/api.js; admin.html; analyst.html; auditor.html</t>
+          <t>src/main/resources/static/js/dom.js; FrontendXssDataExposureTest</t>
         </is>
       </c>
     </row>
@@ -13606,17 +13607,17 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Client-side JavaScript exists, but no explicit DOM clobbering defenses or tests were implemented.</t>
+          <t>Frontend code uses explicit declarations and a dedicated GhostReportDom namespace for rendering helpers, but legacy page scripts still expose some top-level functions, so DOM clobbering hardening is partial.</t>
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>N/A – frontend/browser functionality not in current system scope</t>
+          <t>src/main/resources/static/js/dom.js; src/main/resources/static/js/*.js</t>
         </is>
       </c>
     </row>
@@ -13882,12 +13883,12 @@
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>HSTS is configured with one-year max-age and includeSubDomains, but tests do not assert HSTS on HTTPS responses.</t>
+          <t>Spring Security config sets HSTS max-age 1 year, includeSubDomains and preload for HTTPS responses.</t>
         </is>
       </c>
       <c r="H15" s="16" t="inlineStr">
@@ -13962,17 +13963,17 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
-          <t>CSP is configured with default-src self, object-src none, and frame-ancestors none, but base-uri none is missing and unsafe-inline is allowed.</t>
+          <t>CSP now includes default-src 'self', script-src 'self', object-src 'none', frame-ancestors 'none', base-uri 'none', form-action 'self' and upgrade-insecure-requests, without unsafe-inline/unsafe-eval.</t>
         </is>
       </c>
       <c r="H17" s="16" t="inlineStr">
         <is>
-          <t>SecurityConfig.java; No CorsConfigurationSource implemented</t>
+          <t>SecurityConfig.java; SecurityHeadersTest; FrontendXssDataExposureTest</t>
         </is>
       </c>
     </row>
@@ -14162,17 +14163,17 @@
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G22" s="16" t="inlineStr">
         <is>
-          <t>Cross-Origin-Opener-Policy is not configured for document-rendering responses.</t>
+          <t>COOP, COEP and CORP are configured and asserted for rendered public pages.</t>
         </is>
       </c>
       <c r="H22" s="21" t="inlineStr">
         <is>
-          <t>No implementation evidence found</t>
+          <t>SecurityConfig.java; SecurityHeadersTest</t>
         </is>
       </c>
     </row>
@@ -14220,17 +14221,17 @@
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>CSRF is disabled and authenticated operations use Bearer Authorization headers, but no Origin, Referer, or Sec-Fetch validation is implemented or documented.</t>
+          <t>Unsafe cross-site requests are rejected using Sec-Fetch-Site/Origin validation before controller handling, in addition to Bearer authentication and RBAC.</t>
         </is>
       </c>
       <c r="H24" s="16" t="inlineStr">
         <is>
-          <t>SecurityConfig.java; admin.html; analyst.html; auditor.html</t>
+          <t>SecurityConfig.java; SecurityHeadersTest</t>
         </is>
       </c>
     </row>
@@ -14501,17 +14502,17 @@
       </c>
       <c r="F31" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G31" s="21" t="inlineStr">
         <is>
-          <t>Frame embedding is restricted, and authenticated resources require Bearer/RBAC, but no Sec-Fetch validation or Cross-Origin-Resource-Policy header is configured.</t>
+          <t>Authenticated resources require Bearer/RBAC and cross-origin loading is restricted with Sec-Fetch validation plus Cross-Origin-Resource-Policy same-origin.</t>
         </is>
       </c>
       <c r="H31" s="21" t="inlineStr">
         <is>
-          <t>SecurityConfig.java; ReportService.java; AdminBackupController.java</t>
+          <t>SecurityConfig.java; SecurityHeadersTest; AUTHORIZATION_MATRIX.md</t>
         </is>
       </c>
     </row>
@@ -14998,17 +14999,17 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>The application does not read X-Forwarded-*, X-Real-IP, or X-User-ID headers directly, but no explicit proxy/intermediary header trust policy or tests were implemented.</t>
+          <t>Application code does not trust user-supplied X-Forwarded/X-Real-IP/X-User-ID headers directly; production reverse-proxy mode requires framework/native forwarded-header handling plus explicit trusted-proxy enablement.</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>ReportController.java; SecurityConfig.java; No ForwardedHeaderFilter or forward-headers-strategy implemented</t>
+          <t>SecurityConfigurationValidator.java; application-prod.yaml; SecurityConfigurationValidatorTest</t>
         </is>
       </c>
     </row>
@@ -15136,17 +15137,17 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>Request boundary handling appears to rely on Spring Boot embedded server defaults; no explicit request smuggling protection, proxy configuration, or tests were found.</t>
+          <t>Spring/Tomcat performs HTTP message framing and the application now adds request boundary controls for unsupported TRACE, oversized Authorization/header values, and malformed header characters. External proxy framing remains a deployment control.</t>
         </is>
       </c>
       <c r="H9" s="16" t="inlineStr">
         <is>
-          <t>pom.xml; application.yaml</t>
+          <t>SecurityConfig.java; SecurityHeadersTest; application.yaml; application-prod.yaml</t>
         </is>
       </c>
     </row>
@@ -15176,17 +15177,17 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>The application does not manually set Content-Length and relies on Spring/Tomcat response framing, but no tests or explicit configuration verify conflicting framing is prevented.</t>
+          <t>Application code does not manually construct conflicting Content-Length values and relies on Spring/Tomcat response framing; downloads use framework response entities/content disposition handling.</t>
         </is>
       </c>
       <c r="H10" s="21" t="inlineStr">
         <is>
-          <t>ReportService.java; AdminBackupController.java; No manual Content-Length evidence</t>
+          <t>AdminBackupController.java; ReportController.java; SecurityConfig.java</t>
         </is>
       </c>
     </row>
@@ -15256,17 +15257,17 @@
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>Header values are mostly constants or built with Spring ContentDisposition, but CR/LF header injection rejection is not explicitly configured or tested.</t>
+          <t>Request boundary filter rejects header names/values containing control characters, including CR/LF-style injection attempts before controller handling.</t>
         </is>
       </c>
       <c r="H12" s="21" t="inlineStr">
         <is>
-          <t>SecurityConfig.java; ReportService.java; AdminBackupController.java</t>
+          <t>SecurityConfig.java; SecurityHeadersTest</t>
         </is>
       </c>
     </row>
@@ -15296,17 +15297,17 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr">
         <is>
-          <t>Multipart size limits and file size checks exist, but URI/header length limits and Authorization header size limits are not configured or tested.</t>
+          <t>Server header size and application Authorization/header value limits are configured/tested, reducing oversized-header DoS and malformed request handling risk.</t>
         </is>
       </c>
       <c r="H13" s="16" t="inlineStr">
         <is>
-          <t>application.yaml; FileStorageService.java; RateLimiterService.java</t>
+          <t>application.yaml; application-prod.yaml; SecurityConfig.java; SecurityHeadersTest</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: improve ASVS L2 evidence across chapters
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
+++ b/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
@@ -1468,7 +1468,7 @@
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 266/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls plus CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation.</t>
+          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 267/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls plus CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation and report-submission rate limiting.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -1479,7 +1479,6 @@
       <c r="M3" s="1" t="n"/>
       <c r="O3" s="1" t="n"/>
     </row>
-    <row r="4"/>
     <row r="5" ht="32.1" customHeight="1" s="35">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -3504,17 +3503,17 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="40" t="inlineStr">
         <is>
-          <t>Token type/audience constraints are partly implicit in the application; explicit audience validation remains a limitation.</t>
+          <t>JWTs include explicit iss/aud/jti/type-equivalent header checks and are accepted only after signature, issuer, audience and role validation.</t>
         </is>
       </c>
       <c r="H8" s="40" t="inlineStr">
         <is>
-          <t>JwtService.java; PHASE2_SPRINT2_REPORT.md</t>
+          <t>JwtService.java; JwtServiceSecurityTest</t>
         </is>
       </c>
     </row>
@@ -3544,17 +3543,17 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>JWT audience claims are not issued or validated, so tokens are not restricted to an intended service audience.</t>
+          <t>JWT audience is issued as ghostreport-api and tokens with another audience are rejected even with a valid signature.</t>
         </is>
       </c>
       <c r="H9" s="16" t="inlineStr">
         <is>
-          <t>JwtService.java;</t>
+          <t>JwtService.java; JwtServiceSecurityTest</t>
         </is>
       </c>
     </row>
@@ -3584,17 +3583,17 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>The same configured JWT signing secret is used without audience-restricted tokens because no aud claim is issued.</t>
+          <t>JWTs include an audience claim and key id; current and previous signing keys are scoped through configured kid values for rotation.</t>
         </is>
       </c>
       <c r="H10" s="16" t="inlineStr">
         <is>
-          <t>JwtService.java;</t>
+          <t>JwtService.java; JwtServiceSecurityTest; application.yaml</t>
         </is>
       </c>
     </row>
@@ -5374,17 +5373,17 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>Cryptographic controls (hashing, TLS, token generation) are required by design, but specific algorithms, key management practices, and implementation details are not yet formally defined in Phase 1.</t>
+          <t>JWT and backup HMAC keys have key identifiers and rotation hooks, but an external KMS/vault lifecycle with owner, rotation schedule and destruction workflow is not implemented.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.3 RS8; §2.2 Assumptions (TLS); §11 hashing of codes/files</t>
+          <t>JwtService.java; BackupService.java; SECURE_INSTALLATION.md</t>
         </is>
       </c>
     </row>
@@ -5592,17 +5591,17 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G9" s="21" t="inlineStr">
         <is>
-          <t>Some crypto parameters are configurable, such as JWT secret and expiration, but algorithm agility, key rotation and password hash parameter policy are not implemented or documented.</t>
+          <t>Crypto-relevant keys are externally configured with active/previous JWT kid support and backup HMAC key id, allowing controlled rotation without code changes.</t>
         </is>
       </c>
       <c r="H9" s="21" t="inlineStr">
         <is>
-          <t>application.yaml; JwtService.java; SecurityConfig.java</t>
+          <t>JwtService.java; BackupService.java; SecurityConfigurationValidator.java</t>
         </is>
       </c>
     </row>
@@ -5850,17 +5849,17 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
-          <t>Cryptographic primitives should be selected safely in implementation; exact algorithms are not yet specified.</t>
+          <t>Integrity-sensitive data is protected with HMAC/hashes: JWT HMAC signatures, backup manifest HMAC, audit/security integrity hashes and package hash verification.</t>
         </is>
       </c>
       <c r="H16" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.3 RS8; §2.2 Assumptions (HTTPS/TLS)</t>
+          <t>JwtService.java; BackupService.java; AuditLogService.java; SecurityMonitoringService.java; CasePackageService.java</t>
         </is>
       </c>
     </row>
@@ -7338,17 +7337,17 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>Service-to-service authentication is expected to use least-privilege credentials (e.g., scoped tokens or service accounts), but the exact authentication mechanisms and credential lifecycle are not yet defined.</t>
+          <t>Backend components use externally supplied database credentials and application secrets; there are no unauthenticated backend service integrations in the current single-service design.</t>
         </is>
       </c>
       <c r="H8" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §9 trust boundaries; §10 STRIDE (T/S); §11 mitigations</t>
+          <t>application.yaml; SecurityConfigurationValidator.java; SECURE_INSTALLATION.md</t>
         </is>
       </c>
     </row>
@@ -7458,17 +7457,17 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="21" t="inlineStr">
         <is>
-          <t>Outbound/network/file-access allowlists would strengthen SSRF and egress control but are not yet documented.</t>
+          <t>The application has no user-driven outbound HTTP clients; filesystem access is constrained to configured upload/backup roots with path traversal checks.</t>
         </is>
       </c>
       <c r="H11" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §9 trust boundaries; §10 STRIDE (T/S); §11 mitigations</t>
+          <t>FileStorageService.java; BackupService.java; CasePackageService.java; rg no outbound HTTP clients</t>
         </is>
       </c>
     </row>
@@ -7498,17 +7497,17 @@
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>Outbound/network/file-access allowlists would strengthen SSRF and egress control but are not yet documented.</t>
+          <t>Server-side file access is allowlisted to configured storage roots and safe relative paths; no external URL loading or proxying functionality is implemented.</t>
         </is>
       </c>
       <c r="H12" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §9 trust boundaries; §10 STRIDE (T/S); §11 mitigations</t>
+          <t>FileStorageService.java; BackupService.java; SecurityConfigurationValidator.java</t>
         </is>
       </c>
     </row>
@@ -8195,17 +8194,17 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>Access controls, hashing and integrity checks protect some sensitive data, but protection requirements by classification level are not documented.</t>
+          <t>Sensitive data handling requirements are documented and implemented for JWTs, tracking codes, passwords, uploads, audit logs, backups and evidence packages.</t>
         </is>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>SecurityConfig.java; ReportService.java; BackupService.java; AuditorAuthorizationTest</t>
+          <t>PHASE2_SPRINT2_REPORT.md; SECURITY_ASSESSMENT.md; SECURITY_TESTING.md</t>
         </is>
       </c>
     </row>
@@ -8293,17 +8292,17 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G7" s="21" t="inlineStr">
         <is>
-          <t>SecurityHeadersTest verifies no-store on a static page, but server-side cache/purge behavior for sensitive API responses, backups and generated evidence is not documented.</t>
+          <t>Sensitive API/report/admin/analyst/audit/auth responses receive no-store/no-cache headers, and download responses set no-store headers explicitly.</t>
         </is>
       </c>
       <c r="H7" s="21" t="inlineStr">
         <is>
-          <t>SecurityHeadersTest; BackupService.java; CasePackageService.java</t>
+          <t>SecurityConfig.java; ReportService.java; SecurityHeadersTest; ReportControllerAttachmentUploadTest</t>
         </is>
       </c>
     </row>
@@ -8671,17 +8670,17 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
-          <t>Client-side data protection mechanisms (cache-control headers, storage policies, and token handling) are not yet defined and will be specified if a browser-based UI is introduced.</t>
+          <t>Frontend tests verify bearer tokens are not stored in localStorage/sessionStorage and tracking codes are not placed in URLs; XSRF cookie is not an auth secret.</t>
         </is>
       </c>
       <c r="H17" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.2 RS4-RS6; AC1/AC2; STRIDE P1/P4; §12 tests</t>
+          <t>FrontendXssDataExposureTest; CsrfCookieAttributesTest; js/api.js</t>
         </is>
       </c>
     </row>
@@ -8892,17 +8891,17 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Resource-demanding features are partially identifiable through uploads, backups and rate limits, but anti-availability-loss controls are not fully documented.</t>
+          <t>Resource-demanding functionality is identified and bounded: report creation, uploads/downloads, tracking, login, backups, packages, Hikari pool and Tomcat connection/thread limits.</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>application.yaml; RateLimiterService.java; FileStorageService.java; BackupService.java</t>
+          <t>SECURE_INSTALLATION.md; application.yaml; RateLimiterService.java; BackupService.java</t>
         </is>
       </c>
     </row>
@@ -9070,17 +9069,17 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G10" s="21" t="inlineStr">
         <is>
-          <t>Rate limits, multipart limits and file-size checks reduce availability risk, but backup/package resource limits and broader DoS controls are incomplete.</t>
+          <t>Availability defenses include per-flow rate limits, report submission throttling, upload count/size/type checks, request header limits, Hikari/Tomcat resource limits and controlled backup validation.</t>
         </is>
       </c>
       <c r="H10" s="21" t="inlineStr">
         <is>
-          <t>RateLimiterService.java; RateLimiterServiceTest; application.yaml; FileStorageService.java</t>
+          <t>RateLimiterService.java; ReportController.java; SecurityConfig.java; application.yaml; FileStorageService.java</t>
         </is>
       </c>
     </row>
@@ -9110,17 +9109,17 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>Production config disables H2 console, seed users and stack traces, but no deployment artifact evidence proves test/dev functionality is excluded.</t>
+          <t>Production-like configuration disables H2 console/seed users/dev secrets/stack traces and validates TLS/proxy/resource settings at startup.</t>
         </is>
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
-          <t>application.yaml; application-dev.yaml; DataInitializer.java; DataInitializerDisabledTest</t>
+          <t>application.yaml; application-prod.yaml; SecurityConfigurationValidator.java; DataInitializerDisabledTest</t>
         </is>
       </c>
     </row>
@@ -9368,17 +9367,17 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Rate limiting uses HttpServletRequest.getRemoteAddr, but no trusted proxy/header policy for original client IP was found.</t>
+          <t>Reverse-proxy deployments must opt in to framework/native forwarded-header processing and trusted-proxy mode; otherwise the app uses servlet remote address directly.</t>
         </is>
       </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
-          <t>ReportController.java; No trusted proxy header policy found</t>
+          <t>SecurityConfigurationValidator.java; application-prod.yaml; SecurityConfigurationValidatorTest</t>
         </is>
       </c>
     </row>
@@ -9906,17 +9905,17 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G6" s="21" t="inlineStr">
         <is>
-          <t>Audit timestamps use LocalDateTime without explicit UTC or offset; only some services use Instant/UTC for counters.</t>
+          <t>Audit/security timestamps are generated from Instant in UTC and error responses use ISO-8601 Instant timestamps.</t>
         </is>
       </c>
       <c r="H6" s="21" t="inlineStr">
         <is>
-          <t>AuditLog.java; SecurityAlert.java; RateLimiterService.java</t>
+          <t>AuditLogService.java; SecurityMonitoringService.java; AuditLog.java; SecurityAlert.java; GlobalExceptionHandler.java</t>
         </is>
       </c>
     </row>
@@ -9986,17 +9985,17 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="21" t="inlineStr">
         <is>
-          <t>Logs are structured as JPA entities, but no common external log format, request correlation id or log processor integration was found.</t>
+          <t>Security events are structured JPA entities with correlation id, actor, action/type, target metadata, sanitized details and integrity hash; APIs expose DTOs for review.</t>
         </is>
       </c>
       <c r="H8" s="21" t="inlineStr">
         <is>
-          <t>AuditLog.java; SecurityAlert.java; AuditController.java</t>
+          <t>AuditLog.java; SecurityAlert.java; AuditLogService.java; SecurityMonitoringService.java; AuditController.java</t>
         </is>
       </c>
     </row>
@@ -10204,17 +10203,17 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G14" s="41" t="inlineStr">
         <is>
-          <t>Unexpected/security-sensitive errors are handled generically; external backend TLS failure logging is outside local evidence.</t>
+          <t>Unexpected errors are centrally audited and converted to security alerts while responses remain generic.</t>
         </is>
       </c>
       <c r="H14" s="41" t="inlineStr">
         <is>
-          <t>GlobalExceptionHandler.java; runtime-endpoints.md</t>
+          <t>GlobalExceptionHandler.java; SecurityMonitoringService.java; GlobalExceptionHandlerTest</t>
         </is>
       </c>
     </row>
@@ -10440,17 +10439,17 @@
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G21" s="41" t="inlineStr">
         <is>
-          <t>Controlled errors and backup/attachment validation are evidenced; full external-resource resilience is production dependent.</t>
+          <t>External/resource failures are handled with controlled errors for uploads, backups, packages and malformed runtime requests without exposing stack traces or paths.</t>
         </is>
       </c>
       <c r="H21" s="41" t="inlineStr">
         <is>
-          <t>runtime-endpoints.md</t>
+          <t>GlobalExceptionHandler.java; BackupService.java; FileStorageService.java; runtime-endpoints.md</t>
         </is>
       </c>
     </row>
@@ -11260,7 +11259,7 @@
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>mvn test: 266 tests, 0 failures, 0 errors, 0 skipped.</t>
+          <t>mvn test: 267 tests, 0 failures, 0 errors, 0 skipped.</t>
         </is>
       </c>
     </row>
@@ -11305,7 +11304,7 @@
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>Sprint 2 code hardening added after ASVS review: MFA challenge max-attempt lockout, service-level password policy checks, centralized no-store/no-cache headers, strict CSP/HSTS/CORP/COOP/COEP headers, Fetch Metadata/Origin validation, request header boundary checks, production TLS/verified PostgreSQL TLS validation, and resource-limit validation.</t>
+          <t>Sprint 2 code hardening added after ASVS review: MFA challenge max-attempt lockout, service-level password policy checks, centralized no-store/no-cache headers, strict CSP/HSTS/CORP/COOP/COEP headers, Fetch Metadata/Origin validation, request header boundary checks, production TLS/verified PostgreSQL TLS validation, resource-limit validation, and report-submission rate limiting.</t>
         </is>
       </c>
     </row>
@@ -12873,17 +12872,17 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G5" s="40" t="inlineStr">
         <is>
-          <t>Important limits are documented and tested, but some operational production thresholds remain configuration-dependent.</t>
+          <t>Business limits are documented/configured for report creation, tracking verification, upload, download, login/MFA, file counts/sizes and resource pools.</t>
         </is>
       </c>
       <c r="H5" s="40" t="inlineStr">
         <is>
-          <t>SECURE_INSTALLATION.md; DEVSECOPS_PIPELINE.md</t>
+          <t>application.yaml; RateLimitProperties.java; SECURE_INSTALLATION.md; SECURITY_TESTING.md</t>
         </is>
       </c>
     </row>
@@ -13109,17 +13108,17 @@
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G12" s="21" t="inlineStr">
         <is>
-          <t>Some business limits are implemented for file size/type, rate-limited tracking/upload/download, backup filename format, and closed-case immutability, but report creation, login, listing, backup frequency, and attachment count limits are incomplete.</t>
+          <t>Business limits are implemented for public report submission, tracking, uploads/downloads, login attempts, MFA attempts, file count/size/type and closed-case workflow.</t>
         </is>
       </c>
       <c r="H12" s="21" t="inlineStr">
         <is>
-          <t>RateLimiterService.java; application.yaml; FileStorageService.java; BackupService.java; ClosedCaseSecurityTest; RateLimiterServiceTest</t>
+          <t>RateLimiterService.java; ReportController.java; MfaChallengeService.java; FileStorageService.java; BusinessLogicWorkflowSecurityTest</t>
         </is>
       </c>
     </row>
@@ -13189,17 +13188,17 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="G14" s="21" t="inlineStr">
         <is>
-          <t>Not applicable in the current system design.</t>
+          <t>Not applicable because GhostReport has no limited-quantity inventory such as seats, stock, bookings or quota allocation that can be reserved concurrently.</t>
         </is>
       </c>
       <c r="H14" s="21" t="inlineStr">
         <is>
-          <t>N/A – not in current system scope</t>
+          <t>Architecture scope; ReportService.java</t>
         </is>
       </c>
     </row>
@@ -13287,17 +13286,17 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G17" s="40" t="inlineStr">
         <is>
-          <t>Runtime probes cover repeated invalid tracking/login attempts; production-grade distributed anti-automation remains a limitation.</t>
+          <t>Anti-automation controls cover public report submission, tracking-code verification, upload/download and login brute-force paths; distributed rate limiting remains a production hardening item.</t>
         </is>
       </c>
       <c r="H17" s="40" t="inlineStr">
         <is>
-          <t>runtime-endpoints.md; IAST_RUNTIME_SECURITY.md</t>
+          <t>RateLimiterService.java; ReportController.java; LoginRateLimitSecurityTest; RateLimiterServiceTest</t>
         </is>
       </c>
     </row>
@@ -16249,17 +16248,17 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>No antivirus or malware scanning integration was implemented; existing MIME, extension and magic-byte checks reduce risk but do not provide malware scanning.</t>
+          <t>Uploads are scanned through the MalwareScanner interface; the local implementation detects EICAR, rejects/quarantines malicious uploads and records security alerts.</t>
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr">
         <is>
-          <t>FileStorageService.java; ReportControllerAttachmentUploadTest; No antivirus integration implemented</t>
+          <t>LocalMalwareScanner.java; FileStorageService.java; FileStorageServiceTest; LocalMalwareScannerTest</t>
         </is>
       </c>
     </row>
@@ -16887,17 +16886,17 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>Password handling requirements for internal users are in scope, but these controls are not explicitly defined in the design.</t>
+          <t>The application does not force periodic password expiry; passwords change through user/admin reset/change flows or when policy validation rejects compromised/reused values.</t>
         </is>
       </c>
       <c r="H16" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §6.1 RS2; §6.3 RS10</t>
+          <t>PasswordPolicyService.java; PasswordPolicyAndResetSecurityTest</t>
         </is>
       </c>
     </row>
@@ -16967,17 +16966,17 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Password handling requirements for internal users are in scope, but these controls are not explicitly defined in the design.</t>
+          <t>Password changes and resets are checked against a compromised-password denylist plus reuse/context checks before the new password is accepted.</t>
         </is>
       </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §6.1 RS2; §6.3 RS12</t>
+          <t>PasswordPolicyService.java; PasswordPolicyServiceTest; PasswordPolicyAndResetSecurityTest</t>
         </is>
       </c>
     </row>
@@ -17621,17 +17620,17 @@
       </c>
       <c r="F36" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>MFA codes are one-time: successful verification removes the challenge, expired challenges are removed, and reuse is rejected.</t>
         </is>
       </c>
       <c r="H36" s="16" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>MfaChallengeService.java; AdminMfaAuthenticationTest</t>
         </is>
       </c>
     </row>
@@ -17661,17 +17660,17 @@
       </c>
       <c r="F37" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G37" s="21" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>Short MFA lookup codes are stored only as BCrypt hashes bound to the challenge id; plaintext exposure is limited to dev/test when explicitly enabled.</t>
         </is>
       </c>
       <c r="H37" s="21" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>MfaChallengeService.java; application-prod.yaml; AdminMfaAuthenticationTest</t>
         </is>
       </c>
     </row>
@@ -17701,17 +17700,17 @@
       </c>
       <c r="F38" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G38" s="16" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>MFA codes are generated with SecureRandom, have a configurable TTL and are invalidated after too many wrong attempts.</t>
         </is>
       </c>
       <c r="H38" s="16" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>MfaChallengeService.java; MfaProperties.java; AdminMfaAuthenticationTest</t>
         </is>
       </c>
     </row>
@@ -17999,17 +17998,17 @@
       </c>
       <c r="F46" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G46" s="21" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>MFA verification is bound to the original challenge id and user; the hash input includes challenge id plus code and returns the stored username only after successful verification.</t>
         </is>
       </c>
       <c r="H46" s="21" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>MfaChallengeService.java; AuthService.java; AdminMfaAuthenticationTest</t>
         </is>
       </c>
     </row>
@@ -18275,17 +18274,17 @@
       </c>
       <c r="F54" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G54" s="21" t="inlineStr">
         <is>
-          <t>Application JWTs are HMAC-signed and signature/expiry are checked before authentication, but tampered/expired JWT rejection tests were not found.</t>
+          <t>JWT validation checks HMAC signature, kid, issuer, audience, expiry, jti, subject, role and revocation state before authentication succeeds.</t>
         </is>
       </c>
       <c r="H54" s="21" t="inlineStr">
         <is>
-          <t>JwtService.java; JwtAuthenticationFilter.java; SecurityConfig.java</t>
+          <t>JwtService.java; JwtAuthenticationFilter.java; JwtServiceSecurityTest</t>
         </is>
       </c>
     </row>
@@ -18496,17 +18495,17 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>Session tokens with expiration are defined in the design, but inactivity timeout and absolute maximum lifetime values are not explicitly specified.</t>
+          <t>Session lifetime is stateless JWT based and documented/configured through JWT_EXPIRATION_SECONDS; tokens expire absolutely and revoked tokens are rejected.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>application.yaml; application-dev.yaml; JwtService.java</t>
+          <t>application.yaml; JwtService.java; JwtRevocationPersistenceIntegrationTest; SECURITY_TESTING.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: improve ASVS L3 evidence across chapters
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
+++ b/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
@@ -1468,7 +1468,7 @@
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 267/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls plus CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation and report-submission rate limiting.</t>
+          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 269/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, and CSP violation reporting.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -3046,17 +3046,17 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G14" s="41" t="inlineStr">
         <is>
-          <t>Role/user changes are protected by admin endpoints; immediate revocation semantics are partially evidenced.</t>
+          <t>Admin user deactivation/role-state changes are enforced during JWT validation because current UserDetails account state is checked on each request; disabled users are rejected immediately even with a previously issued token.</t>
         </is>
       </c>
       <c r="H14" s="41" t="inlineStr">
         <is>
-          <t>AdminUserController.java; SECURITY_TESTING.md</t>
+          <t>JwtService.java; JwtAuthenticationFilter.java; AdminUserManagementSecurityTest; UserService.java</t>
         </is>
       </c>
     </row>
@@ -5671,17 +5671,17 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="21" t="inlineStr">
         <is>
-          <t>BCrypt verification is delegated to Spring Security, but custom JWT signature comparison uses String.equals and no constant-time verification evidence was found.</t>
+          <t>JWT signatures are verified using server-side HMAC SHA-256 and MessageDigest.isEqual for constant-time comparison of expected and supplied signatures.</t>
         </is>
       </c>
       <c r="H11" s="21" t="inlineStr">
         <is>
-          <t>JwtService.java; SecurityConfig.java</t>
+          <t>JwtService.java; JwtServiceSecurityTest</t>
         </is>
       </c>
     </row>
@@ -8013,17 +8013,17 @@
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
-          <t>Uploaded files are stored outside static resources and static assets are limited to project files, but no explicit web-tier extension allowlist was found.</t>
+          <t>User uploads are stored outside static resources, filenames are normalized, and the web tier only permits explicit public HTML pages plus /css/** and /js/** static assets; other endpoints remain authenticated/authorized.</t>
         </is>
       </c>
       <c r="H26" s="16" t="inlineStr">
         <is>
-          <t>FileStorageService.java; SecurityConfig.java; src/main/resources/static</t>
+          <t>SecurityConfig.java; FileStorageService.java; SafeFilename.java; SecurityHeadersTest</t>
         </is>
       </c>
     </row>
@@ -8412,17 +8412,17 @@
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Cache-Control no-store is tested for static HTML, but broad web cache deception coverage for authenticated API and download responses is not verified.</t>
+          <t>Sensitive report/auth/admin/analyst/audit/security responses receive no-store/no-cache headers, reducing web cache deception risk for authenticated APIs and downloads.</t>
         </is>
       </c>
       <c r="H10" s="16" t="inlineStr">
         <is>
-          <t>SecurityHeadersTest; SecurityConfig.java; download endpoints</t>
+          <t>SecurityConfig.java; SecurityHeadersTest; ReportController.java; AdminBackupController.java; AnalystController.java</t>
         </is>
       </c>
     </row>
@@ -11178,7 +11178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" style="35" min="1" max="1"/>
@@ -11305,6 +11305,13 @@
       <c r="A20" s="25" t="inlineStr">
         <is>
           <t>Sprint 2 code hardening added after ASVS review: MFA challenge max-attempt lockout, service-level password policy checks, centralized no-store/no-cache headers, strict CSP/HSTS/CORP/COOP/COEP headers, Fetch Metadata/Origin validation, request header boundary checks, production TLS/verified PostgreSQL TLS validation, resource-limit validation, and report-submission rate limiting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Evidence basis: code inspection, tests, Maven output (269 tests, 0 failures, 0 errors, 0 skipped), workflow definitions, runtime probe artefacts and generated security documentation. L3 items that depend on external infrastructure, such as OCSP/ECH, HSM/vault-backed keys or SIEM transport, remain documented as limitations rather than marked compliant.</t>
         </is>
       </c>
     </row>
@@ -11876,17 +11883,17 @@
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="G15" s="21" t="inlineStr">
         <is>
-          <t>CSV/spreadsheet export protection is not implemented or specified. If CSV/XLSX/ODS export is introduced, dangerous leading characters must be escaped.</t>
+          <t>Not applicable in the current GhostReport implementation: no CSV, XLSX or ODS export endpoint exists. Evidence packages/backups use JSON and ZIP artefacts, so spreadsheet formula injection is not currently in scope.</t>
         </is>
       </c>
       <c r="H15" s="21" t="inlineStr">
         <is>
-          <t>Project.pdf: backend API, 3 roles, OS/file ops, ASVS deliverable</t>
+          <t>CasePackageService.java; BackupService.java; no CSV/XLSX/ODS export endpoints</t>
         </is>
       </c>
     </row>
@@ -13468,17 +13475,17 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>Documentation mentions HTTPS/TLS, and Spring Security config implements some browser headers, but expected browser security features and fallback behavior are not fully documented.</t>
+          <t>Browser security expectations are implemented and tested: CSP without unsafe-inline/unsafe-eval, HSTS includeSubDomains/preload, frame denial, no-referrer, Permissions-Policy, COOP/CORP/COEP and no-store for sensitive responses.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>README.md; SecurityConfig.java; SecurityHeadersTest</t>
+          <t>SecurityConfig.java; SecurityHeadersTest; SECURE_INSTALLATION.md; SECURITY_CONFIGURATION_ASSESSMENT.md</t>
         </is>
       </c>
     </row>
@@ -14122,17 +14129,17 @@
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
-          <t>CSP violation reporting is not configured.</t>
+          <t>CSP violation reporting is configured through report-uri /security/csp-report. The endpoint is public/CSRF-exempt for browser reports, stores a sanitized security alert and returns only a generic accepted response.</t>
         </is>
       </c>
       <c r="H21" s="16" t="inlineStr">
         <is>
-          <t>No implementation evidence found</t>
+          <t>SecurityConfig.java; CspReportController.java; SecurityMonitoringService.java; SecurityHeadersTest; SecurityMonitoringServiceTest</t>
         </is>
       </c>
     </row>
@@ -14737,17 +14744,17 @@
       </c>
       <c r="F38" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G38" s="21" t="inlineStr">
         <is>
-          <t>HTTPS is required, but HSTS preload configuration is not defined.</t>
+          <t>HSTS is configured with includeSubDomains, preload and a one-year max-age in Spring Security headers.</t>
         </is>
       </c>
       <c r="H38" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: assumptions §2.2 HTTPS; §5.3 RS7; AC9/AC10</t>
+          <t>SecurityConfig.java; SecurityHeadersTest</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update ASVS L1 L2 L3 evidence
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
+++ b/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
@@ -1468,7 +1468,7 @@
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 269/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, and CSP violation reporting.</t>
+          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 272/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, CSP violation reporting, upload per-report quotas, HTTP parameter pollution rejection and SecureRandom demand tests.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -5769,17 +5769,17 @@
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>Cryptographic primitives should be selected safely in implementation; exact algorithms are not yet specified.</t>
+          <t>No ECB mode or PKCS#1 v1.5 padding usage exists in application cryptography. Implemented primitives are BCrypt, HMAC-SHA256, SHA-256 hashing/integrity and configured TLS cipher suites.</t>
         </is>
       </c>
       <c r="H14" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.3 RS8; §2.2 Assumptions (HTTPS/TLS)</t>
+          <t>JwtService.java; BackupService.java; FileStorageService.java; application-prod.yaml; rg evidence</t>
         </is>
       </c>
     </row>
@@ -5809,17 +5809,17 @@
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G15" s="21" t="inlineStr">
         <is>
-          <t>Cryptographic primitives should be selected safely in implementation; exact algorithms are not yet specified.</t>
+          <t>Application-controlled cryptography uses approved primitives for the implemented scope: BCrypt for passwords, HMAC-SHA256 for JWT/backup integrity, SHA-256 for file/integrity hashes, and modern TLS ciphers in prod-like config.</t>
         </is>
       </c>
       <c r="H15" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.3 RS8; §2.2 Assumptions (HTTPS/TLS)</t>
+          <t>JwtService.java; BackupService.java; FileStorageService.java; application-prod.yaml; PasswordPolicyServiceTest; JwtServiceSecurityTest</t>
         </is>
       </c>
     </row>
@@ -6205,17 +6205,17 @@
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G26" s="21" t="inlineStr">
         <is>
-          <t>SecureRandom is used for tracking codes, but no high-demand randomness or exhaustion tests were found.</t>
+          <t>Tracking codes use a static SecureRandom instance and tests generate 2,000 codes under moderate demand without collisions, supporting randomness behavior under academic load.</t>
         </is>
       </c>
       <c r="H26" s="21" t="inlineStr">
         <is>
-          <t>TrackingCode.java</t>
+          <t>TrackingCode.java; TrackingCodeTest</t>
         </is>
       </c>
     </row>
@@ -6406,12 +6406,12 @@
       </c>
       <c r="G32" s="21" t="inlineStr">
         <is>
-          <t>HSTS is configured and HTTPS/TLS is mentioned, but TLS protocol versions are not explicitly configured or tested in application/deployment files.</t>
+          <t>DTOs, role-specific responses, no-store headers and log redaction minimize exposed data during processing. Encryption-at-rest and immediate post-use encryption for all sensitive data remain operational/future controls.</t>
         </is>
       </c>
       <c r="H32" s="21" t="inlineStr">
         <is>
-          <t>SecurityConfig.java; README.md; application.yaml</t>
+          <t>DTOs; SecurityConfig.java; SecurityLogSanitizer.java; SECURITY_TESTING.md</t>
         </is>
       </c>
     </row>
@@ -7635,17 +7635,17 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>Secrets-management approach should be documented before deployment/implementation.</t>
+          <t>Secrets are externalized through environment/deployment configuration and secret scanning is part of CI. Fine-grained vault/HSM access policies remain future operational work.</t>
         </is>
       </c>
       <c r="H16" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: DFD/trust boundaries §9; STRIDE §10; mitigations §11</t>
+          <t>application.yaml; SECURE_INSTALLATION.md; DEVSECOPS_PIPELINE.md; Gitleaks workflow</t>
         </is>
       </c>
     </row>
@@ -8377,12 +8377,12 @@
       </c>
       <c r="G9" s="21" t="inlineStr">
         <is>
-          <t>RBAC, tracking-code checks, BCrypt, SHA-256 integrity and audit logging exist, but encryption at rest, retention and deletion controls are incomplete.</t>
+          <t>Implemented controls cover RBAC, tracking-code checks, BCrypt, JWT/backup/file integrity, no-store headers, audit/security logging and log redaction. Encryption-at-rest and retention automation remain incomplete.</t>
         </is>
       </c>
       <c r="H9" s="21" t="inlineStr">
         <is>
-          <t>SecurityConfig.java; ReportService.java; BackupService.java; CasePackageService.java</t>
+          <t>SecurityConfig.java; ReportService.java; BackupService.java; CasePackageService.java; SecurityLogSanitizer.java</t>
         </is>
       </c>
     </row>
@@ -9487,17 +9487,17 @@
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G21" s="40" t="inlineStr">
         <is>
-          <t>Runtime negative cases include malformed/wrong content-type inputs; full HTTP parameter pollution review remains partial.</t>
+          <t>HTTP parameter pollution is explicitly rejected for duplicated scalar parameters before controller handling, while multipart uploads remain allowed for file arrays. Runtime and MockMvc tests cover negative behavior.</t>
         </is>
       </c>
       <c r="H21" s="40" t="inlineStr">
         <is>
-          <t>runtime-endpoints.md</t>
+          <t>SecurityConfig.java; SecurityHeadersTest; runtime-endpoints.md</t>
         </is>
       </c>
     </row>
@@ -10341,17 +10341,17 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>Backup and upload failures are logged in selected services, but GlobalExceptionHandler does not log unexpected exceptions or security control failures centrally.</t>
+          <t>GlobalExceptionHandler centrally records unexpected errors in audit logs and security alerts, and security filters/controllers record selected control failures. Secure transmission to a logically separate SIEM remains future operational work.</t>
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: RNF4-RNF5; §5.5 RS12-RS13; AC12; STRIDE D3/P7; §12 tests</t>
+          <t>GlobalExceptionHandler.java; SecurityMonitoringService.java; AuditLogService.java; RuntimeSecurityEventLoggingTest; SECURE_INSTALLATION.md</t>
         </is>
       </c>
     </row>
@@ -11311,7 +11311,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Evidence basis: code inspection, tests, Maven output (269 tests, 0 failures, 0 errors, 0 skipped), workflow definitions, runtime probe artefacts and generated security documentation. L3 items that depend on external infrastructure, such as OCSP/ECH, HSM/vault-backed keys or SIEM transport, remain documented as limitations rather than marked compliant.</t>
+          <t>Evidence basis: code inspection, tests, Maven output (272 tests, 0 failures, 0 errors, 0 skipped), workflow definitions, runtime probe artefacts and generated security documentation. L3 items that depend on external infrastructure, such as OCSP/ECH, HSM/vault-backed keys, SIEM transport, user notification delivery or full session-management UX, remain documented as limitations rather than marked compliant.</t>
         </is>
       </c>
     </row>
@@ -13338,12 +13338,12 @@
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Rate limiting provides partial rapid-call throttling for selected public endpoints, but there is no CAPTCHA-equivalent, realistic human timing control, or rapid repeated report submission protection.</t>
+          <t>Rate limiting throttles rapid login, tracking, download, upload and public report-submission flows. A CAPTCHA/human challenge is not implemented, so this remains partial for L3 human-timing assurance.</t>
         </is>
       </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
-          <t>RateLimiterService.java; ReportController.java; RateLimiterServiceTest; No implementation evidence found for CAPTCHA or human-timing controls</t>
+          <t>RateLimiterService.java; ReportController.java; RateLimiterServiceTest; LoginRateLimitSecurityTest</t>
         </is>
       </c>
     </row>
@@ -15539,17 +15539,17 @@
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>WebSocket session management and token handling are not defined in the design.</t>
+          <t>Not applicable ? the application does not use WebSocket communication or WebSocket session tokens.</t>
         </is>
       </c>
       <c r="H20" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: DFD/trust boundaries §9; STRIDE §10; mitigations §11</t>
+          <t>pom.xml; no WebSocket endpoints/dependencies</t>
         </is>
       </c>
     </row>
@@ -15899,17 +15899,17 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G8" s="41" t="inlineStr">
         <is>
-          <t>Size and type controls are implemented; production quota policy remains partially operational/configuration dependent.</t>
+          <t>Upload size, max files per request and max files per report are enforced. The cumulative per-report quota prevents a single anonymous report from filling storage through repeated upload requests.</t>
         </is>
       </c>
       <c r="H8" s="41" t="inlineStr">
         <is>
-          <t>application*.properties; FileStorageService.java</t>
+          <t>application.yaml; ReportController.java; ReportService.java; AttachmentRepository.java; ReportControllerAttachmentUploadTest; FileStorageService.java</t>
         </is>
       </c>
     </row>
@@ -17071,17 +17071,17 @@
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G21" s="41" t="inlineStr">
         <is>
-          <t>Seed/internal users exist for dev/test evidence; production deployment must replace/disable default credentials.</t>
+          <t>Default/seed users are disabled by default and production-like startup rejects enabled seed users. Test/dev data is explicitly scoped to non-production evidence.</t>
         </is>
       </c>
       <c r="H21" s="41" t="inlineStr">
         <is>
-          <t>data seed/config; SECURE_INSTALLATION.md</t>
+          <t>application.yaml; DataInitializer.java; SecurityConfigurationValidator.java; SecurityConfigurationValidatorTest; DataInitializerDisabledTest</t>
         </is>
       </c>
     </row>
@@ -17489,17 +17489,17 @@
       </c>
       <c r="F32" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G32" s="21" t="inlineStr">
         <is>
-          <t>MFA recovery is not applicable because MFA is not defined in the current design.</t>
+          <t>MFA is implemented for internal roles, but there is no identity-proofed recovery workflow for lost MFA factors. Current academic flow relies on admin/user lifecycle and password reset controls.</t>
         </is>
       </c>
       <c r="H32" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §6.1 RS2-RS3</t>
+          <t>MfaChallengeService.java; AdminMfaAuthenticationTest; PasswordPolicyAndResetSecurityTest; limitation documented</t>
         </is>
       </c>
     </row>
@@ -17529,17 +17529,17 @@
       </c>
       <c r="F33" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G33" s="16" t="inlineStr">
         <is>
-          <t>MFA recovery is not applicable because MFA is not defined in the current design.</t>
+          <t>MFA challenges are short-lived one-time codes, but renewal/reminder workflow for expiring authenticators is not implemented because production MFA delivery remains future work.</t>
         </is>
       </c>
       <c r="H33" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.1 RS1-RS3; AC5/AC8/AC11; STRIDE P5/P6; §12 tests</t>
+          <t>MfaChallengeService.java; AdminMfaAuthenticationTest; SECURE_INSTALLATION.md</t>
         </is>
       </c>
     </row>
@@ -17827,17 +17827,17 @@
       </c>
       <c r="F41" s="18" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G41" s="21" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>Internal user accounts can be disabled and JWTs are rejected when the user is inactive, but there is no separate per-factor revocation inventory for production MFA devices.</t>
         </is>
       </c>
       <c r="H41" s="21" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>UserService.java; JwtService.java; AdminUserManagementSecurityTest; AuthenticationSecurityIntegrationTest</t>
         </is>
       </c>
     </row>
@@ -17872,12 +17872,12 @@
       </c>
       <c r="G42" s="16" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>Not applicable ? GhostReport does not implement biometric authentication.</t>
         </is>
       </c>
       <c r="H42" s="16" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>No biometric authentication implementation</t>
         </is>
       </c>
     </row>
@@ -17912,12 +17912,12 @@
       </c>
       <c r="G43" s="21" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>Not applicable ? GhostReport uses server-generated one-time MFA challenge codes with server-side TTL, not client TOTP values from an authenticator app.</t>
         </is>
       </c>
       <c r="H43" s="21" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>MfaChallengeService.java; AdminMfaAuthenticationTest</t>
         </is>
       </c>
     </row>
@@ -17970,12 +17970,12 @@
       </c>
       <c r="G45" s="16" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>Not applicable ? GhostReport does not deliver MFA through SMS, phone calls or PSTN.</t>
         </is>
       </c>
       <c r="H45" s="16" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>MfaChallengeService.java; SECURE_INSTALLATION.md</t>
         </is>
       </c>
     </row>
@@ -18090,12 +18090,12 @@
       </c>
       <c r="G48" s="21" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>Not applicable ? GhostReport does not implement push-notification MFA.</t>
         </is>
       </c>
       <c r="H48" s="21" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>No push MFA implementation</t>
         </is>
       </c>
     </row>
@@ -18148,12 +18148,12 @@
       </c>
       <c r="G50" s="16" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>Not applicable ? GhostReport does not use cryptographic authentication assertion certificates such as WebAuthn/FIDO or SAML signing certificates.</t>
         </is>
       </c>
       <c r="H50" s="16" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>No WebAuthn/SAML authentication implementation</t>
         </is>
       </c>
     </row>
@@ -18188,12 +18188,12 @@
       </c>
       <c r="G51" s="21" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>Not applicable ? GhostReport does not use cryptographic-device challenge nonces; MFA uses server-generated one-time numeric codes.</t>
         </is>
       </c>
       <c r="H51" s="21" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>MfaChallengeService.java</t>
         </is>
       </c>
     </row>
@@ -18246,12 +18246,12 @@
       </c>
       <c r="G53" s="16" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>Not applicable ? GhostReport does not support multiple identity providers.</t>
         </is>
       </c>
       <c r="H53" s="16" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>No external IdP/OIDC/SAML implementation</t>
         </is>
       </c>
     </row>
@@ -18326,12 +18326,12 @@
       </c>
       <c r="G55" s="16" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>Not applicable ? GhostReport does not consume SAML assertions.</t>
         </is>
       </c>
       <c r="H55" s="16" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>No SAML implementation</t>
         </is>
       </c>
     </row>
@@ -18366,12 +18366,12 @@
       </c>
       <c r="G56" s="21" t="inlineStr">
         <is>
-          <t>Not applicable – the current authentication design does not include MFA, out-of-band methods, cryptographic assertions, or external identity providers.</t>
+          <t>Not applicable ? GhostReport does not use an external IdP or OIDC authentication-strength claims.</t>
         </is>
       </c>
       <c r="H56" s="21" t="inlineStr">
         <is>
-          <t>N/A – not in current authentication scope</t>
+          <t>No OIDC/IdP implementation</t>
         </is>
       </c>
     </row>
@@ -18956,17 +18956,17 @@
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G16" s="41" t="inlineStr">
         <is>
-          <t>Admin user deactivation exists; broad active-session termination on account lifecycle changes remains partially evidenced.</t>
+          <t>Disabling or deleting an internal user terminates effective access because JWT validation reloads current UserDetails and requires the account to remain enabled/non-locked/non-expired on every protected request.</t>
         </is>
       </c>
       <c r="H16" s="41" t="inlineStr">
         <is>
-          <t>AdminUserController.java; AUTHORIZATION_MATRIX.md</t>
+          <t>JwtService.java; JwtAuthenticationFilter.java; UserService.java; AuthenticationSecurityIntegrationTest; AdminUserManagementSecurityTest</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update ASVS final evidence after hardening
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
+++ b/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
@@ -1468,7 +1468,7 @@
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 272/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, CSP violation reporting, upload per-report quotas, HTTP parameter pollution rejection and SecureRandom demand tests.</t>
+          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 274/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, CSP violation reporting, upload per-report quotas, HTTP parameter pollution rejection, SecureRandom demand tests, browser security fallback checks and HTTP/2/3 connection-specific header rejection.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -11311,7 +11311,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Evidence basis: code inspection, tests, Maven output (272 tests, 0 failures, 0 errors, 0 skipped), workflow definitions, runtime probe artefacts and generated security documentation. L3 items that depend on external infrastructure, such as OCSP/ECH, HSM/vault-backed keys, SIEM transport, user notification delivery or full session-management UX, remain documented as limitations rather than marked compliant.</t>
+          <t>Evidence basis: code inspection, tests, Maven output (274 tests, 0 failures, 0 errors, 0 skipped), workflow definitions, runtime probe artefacts and generated security documentation. L3 items that depend on external infrastructure, such as OCSP/ECH, HSM/vault-backed keys, SIEM transport, user notification delivery or full session-management UX, remain documented as limitations rather than marked compliant.</t>
         </is>
       </c>
     </row>
@@ -12657,17 +12657,17 @@
       </c>
       <c r="F36" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>Parser and encoding consistency is partial; standard parsers are used, but manual JSON and raw URL construction remain.</t>
+          <t>Input parsing and output construction use structured APIs rather than ad-hoc interpreter parsing: Jackson/Bean Validation for JSON DTOs, DOM text node helpers for frontend rendering, URI/path normalization helpers for file paths, and no tracking-code query parsing in the browser.</t>
         </is>
       </c>
       <c r="H36" s="16" t="inlineStr">
         <is>
-          <t>CasePackageService.java; JwtService.java; submit.html; track.html; AdminBackupController.java</t>
+          <t>DTOs; GlobalExceptionHandler.java; SafeFilename.java; TrackingCode.java; dom.js; FrontendXssDataExposureTest</t>
         </is>
       </c>
     </row>
@@ -14784,17 +14784,17 @@
       </c>
       <c r="F39" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G39" s="16" t="inlineStr">
         <is>
-          <t>No browser-specific behavior or fallback mechanisms are defined in the design.</t>
+          <t>Static pages now load /js/security-support.js, which detects missing browser security/runtime features such as fetch, Promise, crypto.getRandomValues, TextEncoder and DOM replacement APIs, then shows a warning and disables interactive controls.</t>
         </is>
       </c>
       <c r="H39" s="16" t="inlineStr">
         <is>
-          <t>Project.pdf: backend API, 3 roles, OS/file ops, ASVS deliverable</t>
+          <t>security-support.js; static HTML pages; style.css; FrontendXssDataExposureTest</t>
         </is>
       </c>
     </row>
@@ -15223,17 +15223,17 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>No manual Transfer-Encoding or connection-specific HTTP/2/HTTP/3 header handling was found, but there is no explicit HTTP/2/3 proxy/server policy or test evidence.</t>
+          <t>HTTP/2 and HTTP/3 requests with connection-specific headers such as Transfer-Encoding, Connection, Upgrade, Keep-Alive or Proxy-Connection are rejected by the request-boundary filter before controller handling.</t>
         </is>
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
-          <t>application.yaml; pom.xml</t>
+          <t>SecurityConfig.java; SecurityHeadersTest</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update ASVS evidence for additional hardening
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
+++ b/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
@@ -1468,7 +1468,7 @@
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 274/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, CSP violation reporting, upload per-report quotas, HTTP parameter pollution rejection, SecureRandom demand tests, browser security fallback checks and HTTP/2/3 connection-specific header rejection.</t>
+          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 281/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, CSP violation reporting, upload per-report quotas, HTTP parameter pollution rejection, SecureRandom demand tests, browser security fallback checks, HTTP/2/3 connection-specific header rejection, composition-free password policy, source-control metadata blocking and cryptographic inventory verification.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -5373,17 +5373,17 @@
       </c>
       <c r="F3" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>JWT and backup HMAC keys have key identifiers and rotation hooks, but an external KMS/vault lifecycle with owner, rotation schedule and destruction workflow is not implemented.</t>
+          <t>A cryptographic inventory and change policy now document current algorithms, key/secret material, ownership and rotation expectations for JWT, backup HMAC, BCrypt, SecureRandom and SHA-256 integrity uses.</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>JwtService.java; BackupService.java; SECURE_INSTALLATION.md</t>
+          <t>CRYPTOGRAPHIC_INVENTORY.md; SECURE_INSTALLATION.md; CryptographicInventoryTest</t>
         </is>
       </c>
     </row>
@@ -5453,17 +5453,17 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Cryptographic controls (hashing, TLS, token generation) are required by design, but specific algorithms, key management practices, and implementation details are not yet formally defined in Phase 1.</t>
+          <t>CryptographicInventoryTest statically scans application source for cryptographic mechanisms and asserts that expected uses are mapped in CRYPTOGRAPHIC_INVENTORY.md.</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.3 RS8; §2.2 Assumptions (TLS); §11 hashing of codes/files</t>
+          <t>CryptographicInventoryTest; CRYPTOGRAPHIC_INVENTORY.md</t>
         </is>
       </c>
     </row>
@@ -5493,17 +5493,17 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G6" s="21" t="inlineStr">
         <is>
-          <t>Cryptographic controls (hashing, TLS, token generation) are required by design, but specific algorithms, key management practices, and implementation details are not yet formally defined in Phase 1.</t>
+          <t>CRYPTOGRAPHIC_INVENTORY.md maintains the cryptographic inventory and records the migration/rotation policy and limitations, including lack of external HSM/vault and post-quantum migration as future work.</t>
         </is>
       </c>
       <c r="H6" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.3 RS8; §2.2 Assumptions (TLS); §11 hashing of codes/files</t>
+          <t>CRYPTOGRAPHIC_INVENTORY.md; ASVS_EVIDENCE.md</t>
         </is>
       </c>
     </row>
@@ -7773,17 +7773,17 @@
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G20" s="40" t="inlineStr">
         <is>
-          <t>Deployment hygiene is documented; repository metadata exclusion is a packaging/deployment responsibility.</t>
+          <t>The request-boundary filter explicitly blocks /.git and /.svn paths with controlled 404 responses, and only named static pages plus /css/** and /js/** are public.</t>
         </is>
       </c>
       <c r="H20" s="40" t="inlineStr">
         <is>
-          <t>SECURE_INSTALLATION.md</t>
+          <t>SecurityConfig.java; SecurityHeadersTest</t>
         </is>
       </c>
     </row>
@@ -11311,7 +11311,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Evidence basis: code inspection, tests, Maven output (274 tests, 0 failures, 0 errors, 0 skipped), workflow definitions, runtime probe artefacts and generated security documentation. L3 items that depend on external infrastructure, such as OCSP/ECH, HSM/vault-backed keys, SIEM transport, user notification delivery or full session-management UX, remain documented as limitations rather than marked compliant.</t>
+          <t>Evidence basis: code inspection, tests, Maven output (281 tests, 0 failures, 0 errors, 0 skipped), workflow definitions, runtime probe artefacts and generated security documentation. L3 items that depend on external infrastructure, such as OCSP/ECH, HSM/vault-backed keys, SIEM transport, user notification delivery or full session-management UX, remain documented as limitations rather than marked compliant.</t>
         </is>
       </c>
     </row>
@@ -16693,17 +16693,17 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>Internal user authentication is in scope, but the password policy is not explicitly defined in the design.</t>
+          <t>Password policy accepts any character composition and no longer requires uppercase/lowercase/digit/symbol classes. Controls remain length limits, compromised-password denylist, context-word rejection and reuse/history checks.</t>
         </is>
       </c>
       <c r="H11" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §6.1 RS2; §6.3 RS12</t>
+          <t>PasswordPolicyService.java; CreateUserRequest.java; ChangePasswordRequest.java; PasswordResetConfirmRequest.java; PasswordPolicyServiceTest; AuthenticationSecurityIntegrationTest</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update ASVS evidence for admin reset and DOM controls
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
+++ b/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
@@ -1468,7 +1468,7 @@
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 281/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, CSP violation reporting, upload per-report quotas, HTTP parameter pollution rejection, SecureRandom demand tests, browser security fallback checks, HTTP/2/3 connection-specific header rejection, composition-free password policy, source-control metadata blocking and cryptographic inventory verification.</t>
+          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 283/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, CSP violation reporting, upload per-report quotas, HTTP parameter pollution rejection, SecureRandom demand tests, browser security fallback checks, HTTP/2/3 connection-specific header rejection, composition-free password policy, source-control metadata blocking, cryptographic inventory verification, admin-initiated password reset and DOM clobbering checks.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -11311,7 +11311,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Evidence basis: code inspection, tests, Maven output (281 tests, 0 failures, 0 errors, 0 skipped), workflow definitions, runtime probe artefacts and generated security documentation. L3 items that depend on external infrastructure, such as OCSP/ECH, HSM/vault-backed keys, SIEM transport, user notification delivery or full session-management UX, remain documented as limitations rather than marked compliant.</t>
+          <t>Evidence basis: code inspection, tests, Maven output (283 tests, 0 failures, 0 errors, 0 skipped), workflow definitions, runtime probe artefacts and generated security documentation. L3 items that depend on external infrastructure, such as OCSP/ECH, HSM/vault-backed keys, SIEM transport, user notification delivery or full session-management UX, remain documented as limitations rather than marked compliant.</t>
         </is>
       </c>
     </row>
@@ -13613,17 +13613,17 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Frontend code uses explicit declarations and a dedicated GhostReportDom namespace for rendering helpers, but legacy page scripts still expose some top-level functions, so DOM clobbering hardening is partial.</t>
+          <t>Frontend tests assert that forms/controls do not use name attributes that can clobber document/window properties, and that JavaScript does not access page elements through document.&lt;id&gt;; DOM access uses explicit lookup/helper APIs.</t>
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>src/main/resources/static/js/dom.js; src/main/resources/static/js/*.js</t>
+          <t>FrontendXssDataExposureTest; dom.js; static HTML pages</t>
         </is>
       </c>
     </row>
@@ -17569,17 +17569,17 @@
       </c>
       <c r="F34" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G34" s="21" t="inlineStr">
         <is>
-          <t>Recovery/reset processes for internal users are possible but not yet specified in detail.</t>
+          <t>Administrators can initiate password reset through POST /admin/users/{id}/password-reset, which issues a reset token through the existing reset flow but never lets the administrator choose or know the new password. The action is audited as PASSWORD_RESET_ADMIN_INITIATED.</t>
         </is>
       </c>
       <c r="H34" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.1 RS1-RS3; AC5/AC8/AC11; STRIDE P5/P6; §12 tests</t>
+          <t>AdminController.java; PasswordResetService.java; AdminUserManagementSecurityTest</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update ASVS evidence for L3 hardening
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
+++ b/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
@@ -1468,7 +1468,7 @@
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 283/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, CSP violation reporting, upload per-report quotas, HTTP parameter pollution rejection, SecureRandom demand tests, browser security fallback checks, HTTP/2/3 connection-specific header rejection, composition-free password policy, source-control metadata blocking, cryptographic inventory verification, admin-initiated password reset and DOM clobbering checks.</t>
+          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 286/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, CSP violation reporting, upload per-report quotas, HTTP parameter pollution rejection, SecureRandom demand tests, browser security fallback checks, HTTP/2/3 connection-specific header rejection, composition-free password policy, source-control metadata blocking, cryptographic inventory verification, admin-initiated password reset, DOM clobbering checks, admin backup restore reauthentication, minimized internal-path API responses and dangerous-functionality inventory verification.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -5889,17 +5889,17 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="G17" s="21" t="inlineStr">
         <is>
-          <t>This is advanced crypto-hardening detail not yet covered in Phase 1 documentation.</t>
+          <t>Not applicable to current application code: GhostReport does not use application-level Cipher/encryption modes with IV/nonces. Current crypto usage is BCrypt, SecureRandom, HMAC-SHA-256, SHA-256 and platform TLS.</t>
         </is>
       </c>
       <c r="H17" s="21" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.3 RS8; §2.2 Assumptions (HTTPS/TLS)</t>
+          <t>CRYPTOGRAPHIC_INVENTORY.md; CryptographicInventoryTest</t>
         </is>
       </c>
     </row>
@@ -5929,17 +5929,17 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Not Applicable</t>
         </is>
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>This is advanced crypto-hardening detail not yet covered in Phase 1 documentation.</t>
+          <t>Not applicable to current application code: GhostReport does not compose encryption and MAC algorithms for encrypted payloads. Backups use HMAC over manifests plus hashes, not encrypt-then-MAC encryption.</t>
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.3 RS8; §2.2 Assumptions (HTTPS/TLS)</t>
+          <t>CRYPTOGRAPHIC_INVENTORY.md; BackupService.java; BackupServiceIntegrationTest</t>
         </is>
       </c>
     </row>
@@ -8452,17 +8452,17 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G11" s="41" t="inlineStr">
         <is>
-          <t>DTOs and role-specific responses minimize exposed fields, but a full data minimization review remains a limitation.</t>
+          <t>API responses were minimized so backup restore and case package generation no longer expose internal restore/package paths or generated file lists; response DTOs are guarded by a minimization test.</t>
         </is>
       </c>
       <c r="H11" s="41" t="inlineStr">
         <is>
-          <t>DTOs; SECURITY_TESTING.md</t>
+          <t>BackupRestoreResponse.java; CasePackageResponse.java; BackupService.java; CasePackageService.java; ResponseDataMinimizationTest</t>
         </is>
       </c>
     </row>
@@ -8971,17 +8971,17 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Dangerous functionality such as file uploads, backup restore and evidence package generation exists and is protected in code, but a documented dangerous-functionality inventory was not found.</t>
+          <t>Dangerous functionality is documented in a dedicated inventory covering backup restore, uploads, downloads, evidence packages, password reset, JWT, logs and crypto, with a test that maps code tokens to documentation.</t>
         </is>
       </c>
       <c r="H7" s="16" t="inlineStr">
         <is>
-          <t>FileStorageService.java; BackupService.java; CasePackageService.java; AdminBackupController.java</t>
+          <t>DANGEROUS_FUNCTIONALITY.md; DangerousFunctionalityInventoryTest</t>
         </is>
       </c>
     </row>
@@ -19214,17 +19214,17 @@
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Compliant</t>
         </is>
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
-          <t>Sensitive-account-operation re-authentication/session management is not yet fully defined.</t>
+          <t>Sensitive actions now require secondary verification where implemented: password change requires current password and admin backup restore requires X-Reauth-Password validated against the authenticated ADMIN before staging restore.</t>
         </is>
       </c>
       <c r="H23" s="16" t="inlineStr">
         <is>
-          <t>DESOFS Phase 1: §5.1 RS1-RS3; AC5/AC8/AC11; STRIDE P5/P6; §12 tests</t>
+          <t>AuthController.java; AdminBackupController.java; ReauthenticationService.java; PasswordPolicyAndResetSecurityTest; AdminBackupControllerSecurityTest</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: document ZAP triage and ASVS evidence
</commit_message>
<xml_diff>
--- a/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
+++ b/Deliverables/Phase 2/Sprint 2/ASVS_5.0_Tracker_Phase_2_Sprint_2.xlsx
@@ -1468,7 +1468,7 @@
     <row r="3" ht="18" customHeight="1" s="35">
       <c r="A3" s="39" t="inlineStr">
         <is>
-          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 286/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, CSP violation reporting, upload per-report quotas, HTTP parameter pollution rejection, SecureRandom demand tests, browser security fallback checks, HTTP/2/3 connection-specific header rejection, composition-free password policy, source-control metadata blocking, cryptographic inventory verification, admin-initiated password reset, DOM clobbering checks, admin backup restore reauthentication, minimized internal-path API responses and dangerous-functionality inventory verification.</t>
+          <t>Updated from Phase 2 Sprint 1 workbook for Sprint 2 evidence: tests 286/0/0/0; runtime probes 101 total, 101 passed, 0 failed, 0 skipped; Dependency-Check 0 unsuppressed vulnerabilities; Sprint 2 hardening added MFA/password/no-cache controls, CSP/HSTS/Fetch Metadata/request-boundary/TLS/resource-limit validation, report-submission rate limiting, CSP violation reporting, upload per-report quotas, HTTP parameter pollution rejection, SecureRandom demand tests, browser security fallback checks, HTTP/2/3 connection-specific header rejection, composition-free password policy, source-control metadata blocking, cryptographic inventory verification, admin-initiated password reset, DOM clobbering checks, admin backup restore reauthentication, minimized internal-path API responses and dangerous-functionality inventory verification. CSP reporting now uses report-to and Report-To header instead of deprecated report-uri.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -1479,6 +1479,7 @@
       <c r="M3" s="1" t="n"/>
       <c r="O3" s="1" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5" ht="32.1" customHeight="1" s="35">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -14134,7 +14135,7 @@
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
-          <t>CSP violation reporting is configured through report-uri /security/csp-report. The endpoint is public/CSRF-exempt for browser reports, stores a sanitized security alert and returns only a generic accepted response.</t>
+          <t>CSP violation reporting is configured through report-to csp-endpoint with Report-To /security/csp-report. The endpoint is public/CSRF-exempt for browser reports, stores a sanitized security alert and returns only a generic accepted response.</t>
         </is>
       </c>
       <c r="H21" s="16" t="inlineStr">

</xml_diff>